<commit_message>
feat: numero de faixas dinamico
</commit_message>
<xml_diff>
--- a/referencias_template.xlsx
+++ b/referencias_template.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucoes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cargos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras_Calculo" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tetos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metas_Mensais" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOTVS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regras_Calculo" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tetos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metas_Mensais" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOTVS" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +66,14 @@
       <i val="1"/>
       <color rgb="00595959"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
     </font>
   </fonts>
   <fills count="7">
@@ -112,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -161,6 +170,10 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -526,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -567,48 +580,48 @@
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Cargos</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Qual grupo de calculo cada cargo pertence. Confirmar os nomes exatos do TOTVS.</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>RH / Gestao</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Grupos</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Se a base do premio de cada grupo e o salario (percentual) ou um teto fixo em R$ (teto_fixo).</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Gestao RV</t>
         </is>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Regras_Calculo</t>
+          <t>Cargos</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Faixas de atingimento e percentuais de premio por grupo e indicador.</t>
+          <t>Qual grupo de calculo cada cargo pertence. Confirmar os nomes exatos do TOTVS.</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Gestao RV</t>
+          <t>RH / Gestao</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Tetos</t>
+          <t>Regras_Calculo</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Valor maximo de premio em R$ por cargo (modelo teto fixo).</t>
+          <t>Faixas de atingimento e percentuais de premio por grupo e indicador.</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -620,12 +633,12 @@
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Metas_Mensais</t>
+          <t>Tetos</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Metas de NPS e NONREV — atualizar todo mes antes de rodar o calculo.</t>
+          <t>Valor maximo de premio em R$ por cargo (modelo teto fixo).</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -637,29 +650,46 @@
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>Metas_Mensais</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Metas de NPS e NONREV — atualizar todo mes antes de rodar o calculo.</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Gestao RV</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>TOTVS</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Codigo do evento e parametros tecnicos de integracao com o TOTVS RM.</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>TI / TOTVS</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Celulas com fundo LARANJA precisam de confirmacao antes do primeiro uso em producao.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Celulas com fundo AZUL CLARO sao linhas em branco para novos registros.</t>
         </is>
@@ -1387,852 +1417,142 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>grupo</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>indicador</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>faixa1_min</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>faixa1_max</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>faixa2_min</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>faixa2_max</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>faixa1_pct</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>faixa2_pct</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>direcao</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
-        <is>
-          <t>chave_meta</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Nome do grupo</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Nome do indicador</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>Minimo faixa 1</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>Maximo faixa 1</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>Minimo faixa 2</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>Maximo faixa 2</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>% faixa 1 (ex: 0,15 = 15%)</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>% faixa 2 (ex: 0,45 = 45%)</t>
-        </is>
-      </c>
-      <c r="I2" s="7" t="inlineStr">
-        <is>
-          <t>maior ou menor</t>
-        </is>
-      </c>
-      <c r="J2" s="7" t="inlineStr">
-        <is>
-          <t>Chave em Metas_Mensais (vazio = limite fixo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Nome do grupo (igual ao usado em Cargos e Regras_Calculo)</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="inlineStr">
+        <is>
+          <t>percentual ou teto_fixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>atendente</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>dma</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="n">
-        <v>38</v>
-      </c>
-      <c r="D3" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="E3" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="F3" s="11" t="n"/>
-      <c r="G3" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H3" s="11" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="I3" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J3" s="11" t="n"/>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>atendente</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>nps</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>74</v>
-      </c>
-      <c r="D4" s="11" t="n">
-        <v>77</v>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>77</v>
-      </c>
-      <c r="F4" s="11" t="n"/>
-      <c r="G4" s="11" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H4" s="11" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I4" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J4" s="11" t="n"/>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>atendente</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>faturamento</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="F5" s="11" t="n"/>
-      <c r="G5" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H5" s="11" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J5" s="11" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>percentual</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>atendente_lider</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>dma</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>38</v>
-      </c>
-      <c r="D6" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="F6" s="11" t="n"/>
-      <c r="G6" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H6" s="11" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="I6" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J6" s="11" t="n"/>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>atendente_lider</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>nps</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="n">
-        <v>74</v>
-      </c>
-      <c r="D7" s="11" t="n">
-        <v>77</v>
-      </c>
-      <c r="E7" s="11" t="n">
-        <v>77</v>
-      </c>
-      <c r="F7" s="11" t="n"/>
-      <c r="G7" s="11" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H7" s="11" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I7" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J7" s="11" t="n"/>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>atendente_lider</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>faturamento</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="D8" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="E8" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="F8" s="11" t="n"/>
-      <c r="G8" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H8" s="11" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="I8" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J8" s="11" t="n"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>percentual</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>gestor</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>dma</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>38</v>
-      </c>
-      <c r="D9" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H9" s="11" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="I9" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J9" s="11" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>gestor</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>nps</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>74</v>
-      </c>
-      <c r="D10" s="11" t="n">
-        <v>77</v>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>77</v>
-      </c>
-      <c r="F10" s="11" t="n"/>
-      <c r="G10" s="11" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H10" s="11" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I10" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J10" s="11" t="n"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>gestor</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>faturamento</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="D11" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H11" s="11" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="I11" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J11" s="11" t="n"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>percentual</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>regional</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>dma</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>38</v>
-      </c>
-      <c r="D12" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H12" s="11" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="I12" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J12" s="11" t="n"/>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>regional</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>nps</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="n">
-        <v>74</v>
-      </c>
-      <c r="D13" s="11" t="n">
-        <v>77</v>
-      </c>
-      <c r="E13" s="11" t="n">
-        <v>77</v>
-      </c>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H13" s="11" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I13" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J13" s="11" t="n"/>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>regional</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>faturamento</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="D14" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="E14" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H14" s="11" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J14" s="11" t="n"/>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>percentual</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>mecanico</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>percentual</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>lider_frota</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>nps</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="n"/>
-      <c r="D15" s="12" t="n"/>
-      <c r="E15" s="12" t="n"/>
-      <c r="F15" s="12" t="n"/>
-      <c r="G15" s="11" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H15" s="11" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="I15" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J15" s="11" t="inlineStr">
-        <is>
-          <t>nps_lider_frota</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>lider_frota</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>preventiva</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n">
-        <v>97</v>
-      </c>
-      <c r="D16" s="11" t="n">
-        <v>99</v>
-      </c>
-      <c r="E16" s="11" t="n">
-        <v>99</v>
-      </c>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H16" s="11" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J16" s="11" t="n"/>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>lider_frota</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>nonrev</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="n"/>
-      <c r="D17" s="12" t="n"/>
-      <c r="E17" s="12" t="n"/>
-      <c r="F17" s="12" t="n"/>
-      <c r="G17" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I17" s="11" t="inlineStr">
-        <is>
-          <t>menor</t>
-        </is>
-      </c>
-      <c r="J17" s="11" t="inlineStr">
-        <is>
-          <t>nonrev</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>teto_fixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>lider_patio</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>nps</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="12" t="n"/>
-      <c r="F18" s="12" t="n"/>
-      <c r="G18" s="11" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H18" s="11" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="I18" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J18" s="11" t="inlineStr">
-        <is>
-          <t>nps_lider_patio</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>lider_patio</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>nonrev</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="12" t="n"/>
-      <c r="E19" s="12" t="n"/>
-      <c r="F19" s="12" t="n"/>
-      <c r="G19" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H19" s="11" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I19" s="11" t="inlineStr">
-        <is>
-          <t>menor</t>
-        </is>
-      </c>
-      <c r="J19" s="11" t="inlineStr">
-        <is>
-          <t>nonrev</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>lider_patio</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>bate_patio</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="F20" s="11" t="n"/>
-      <c r="G20" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="11" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J20" s="11" t="n"/>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>teto_fixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>operador_frota</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>nps</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="n"/>
-      <c r="D21" s="12" t="n"/>
-      <c r="E21" s="12" t="n"/>
-      <c r="F21" s="12" t="n"/>
-      <c r="G21" s="11" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H21" s="11" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="I21" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J21" s="11" t="inlineStr">
-        <is>
-          <t>nps_operador_frota</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>operador_frota</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>preventiva</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="n">
-        <v>97</v>
-      </c>
-      <c r="D22" s="11" t="n">
-        <v>99</v>
-      </c>
-      <c r="E22" s="11" t="n">
-        <v>99</v>
-      </c>
-      <c r="F22" s="11" t="n"/>
-      <c r="G22" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H22" s="11" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I22" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J22" s="11" t="n"/>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>operador_frota</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>nonrev</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="n"/>
-      <c r="D23" s="12" t="n"/>
-      <c r="E23" s="12" t="n"/>
-      <c r="F23" s="12" t="n"/>
-      <c r="G23" s="11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H23" s="11" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I23" s="11" t="inlineStr">
-        <is>
-          <t>menor</t>
-        </is>
-      </c>
-      <c r="J23" s="11" t="inlineStr">
-        <is>
-          <t>nonrev</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>teto_fixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>outros</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>nps</t>
-        </is>
-      </c>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="12" t="n"/>
-      <c r="F24" s="12" t="n"/>
-      <c r="G24" s="11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H24" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I24" s="11" t="inlineStr">
-        <is>
-          <t>maior</t>
-        </is>
-      </c>
-      <c r="J24" s="11" t="inlineStr">
-        <is>
-          <t>nps_outros</t>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>teto_fixo</t>
         </is>
       </c>
     </row>
@@ -2242,6 +1562,1413 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>grupo</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>indicador</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>faixa</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>valor_min</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>valor_max</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="G1" s="18" t="inlineStr">
+        <is>
+          <t>direcao</t>
+        </is>
+      </c>
+      <c r="H1" s="18" t="inlineStr">
+        <is>
+          <t>chave_meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Nome do grupo</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="inlineStr">
+        <is>
+          <t>Nome do indicador</t>
+        </is>
+      </c>
+      <c r="C2" s="19" t="inlineStr">
+        <is>
+          <t>Numero da faixa (1, 2, 3... - maior numero = melhor faixa)</t>
+        </is>
+      </c>
+      <c r="D2" s="19" t="inlineStr">
+        <is>
+          <t>Minimo da faixa</t>
+        </is>
+      </c>
+      <c r="E2" s="19" t="inlineStr">
+        <is>
+          <t>Maximo da faixa (exclusivo)</t>
+        </is>
+      </c>
+      <c r="F2" s="19" t="inlineStr">
+        <is>
+          <t>% credit. nessa faixa (ex: 0,15 = 15%)</t>
+        </is>
+      </c>
+      <c r="G2" s="19" t="inlineStr">
+        <is>
+          <t>maior ou menor</t>
+        </is>
+      </c>
+      <c r="H2" s="19" t="inlineStr">
+        <is>
+          <t>Chave em Metas_Mensais (vazio = limite fixo aqui mesmo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>atendente</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>dma</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>38</v>
+      </c>
+      <c r="E3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>atendente</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>dma</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>40</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>atendente</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>74</v>
+      </c>
+      <c r="E5" t="n">
+        <v>77</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>atendente</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>77</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>atendente</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>faturamento</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" t="n">
+        <v>105</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>atendente</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>faturamento</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>105</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>atendente_lider</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>dma</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>38</v>
+      </c>
+      <c r="E9" t="n">
+        <v>40</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>atendente_lider</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>dma</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>40</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>atendente_lider</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>74</v>
+      </c>
+      <c r="E11" t="n">
+        <v>77</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>atendente_lider</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>77</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>atendente_lider</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>faturamento</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E13" t="n">
+        <v>105</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>atendente_lider</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>faturamento</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" t="n">
+        <v>105</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>gestor</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>dma</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>38</v>
+      </c>
+      <c r="E15" t="n">
+        <v>40</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>gestor</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>dma</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>40</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>gestor</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>74</v>
+      </c>
+      <c r="E17" t="n">
+        <v>77</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>gestor</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>77</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>gestor</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>faturamento</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>100</v>
+      </c>
+      <c r="E19" t="n">
+        <v>105</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>gestor</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>faturamento</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>105</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>regional</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>dma</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>38</v>
+      </c>
+      <c r="E21" t="n">
+        <v>40</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>regional</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>dma</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>40</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>regional</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>74</v>
+      </c>
+      <c r="E23" t="n">
+        <v>77</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>regional</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>77</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>regional</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>faturamento</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>100</v>
+      </c>
+      <c r="E25" t="n">
+        <v>105</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>regional</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>faturamento</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>105</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>lider_frota</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>nps_lider_frota</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>lider_frota</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>nps_lider_frota</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>lider_frota</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>preventiva</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>97</v>
+      </c>
+      <c r="E29" t="n">
+        <v>99</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>lider_frota</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>preventiva</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" t="n">
+        <v>99</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>lider_frota</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>menor</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>lider_frota</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>menor</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>lider_patio</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>nps_lider_patio</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>lider_patio</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>nps_lider_patio</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>lider_patio</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>menor</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>lider_patio</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>menor</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>lider_patio</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>bate_patio</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" t="n">
+        <v>100</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>operador_frota</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>nps_operador_frota</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>operador_frota</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>nps_operador_frota</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>operador_frota</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>preventiva</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>97</v>
+      </c>
+      <c r="E40" t="n">
+        <v>99</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>operador_frota</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>preventiva</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="n">
+        <v>99</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>operador_frota</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>menor</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>operador_frota</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>menor</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>outros</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>nps_outros</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>outros</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>nps</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>nps_outros</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>mecanico</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>preventiva</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>96</v>
+      </c>
+      <c r="E46" t="n">
+        <v>99</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>mecanico</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>preventiva</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>99</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>maior</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>mecanico</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>menor</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>mecanico</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>menor</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2663,382 +3390,284 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>mes</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="18" t="inlineStr">
         <is>
           <t>chave</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>faixa1_min</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>faixa1_max</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>faixa2_min</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>faixa2_max</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="70" customHeight="1">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>AAAA-MM
-ex: 2026-07</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>nps_lider_frota
-nps_lider_patio
-nps_operador_frota
-nps_outros
-nonrev</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>NPS: minimo faixa 1
-NONREV: minimo faixa 1</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>NPS: maximo faixa 1
-NONREV: maximo faixa 1</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>NPS: minimo faixa 2
-NONREV: deixar vazio</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>NONREV: maximo faixa 2
-NPS: deixar vazio</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>faixa</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>valor_min</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>valor_max</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>AAAA-MM (ex: 2026-07)</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="inlineStr">
+        <is>
+          <t>nps_lider_frota / nps_lider_patio / nps_operador_frota / nps_outros / nonrev</t>
+        </is>
+      </c>
+      <c r="C2" s="19" t="inlineStr">
+        <is>
+          <t>Numero da faixa (1, 2...)</t>
+        </is>
+      </c>
+      <c r="D2" s="19" t="inlineStr">
+        <is>
+          <t>Minimo da faixa (NPS) ou vazio na melhor faixa (NONREV)</t>
+        </is>
+      </c>
+      <c r="E2" s="19" t="inlineStr">
+        <is>
+          <t>Maximo da faixa (exclusivo) ou vazio na melhor faixa (NPS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>2026-06</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>nps_lider_frota</t>
         </is>
       </c>
-      <c r="C3" s="15" t="n">
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
         <v>78</v>
       </c>
-      <c r="D3" s="15" t="n">
+      <c r="E3" t="n">
         <v>80</v>
       </c>
-      <c r="E3" s="15" t="n">
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>nps_lider_frota</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
         <v>80</v>
       </c>
-      <c r="F3" s="15" t="n"/>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>2026-06</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>nps_lider_patio</t>
         </is>
       </c>
-      <c r="C4" s="15" t="n">
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
         <v>77</v>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="E5" t="n">
         <v>79</v>
       </c>
-      <c r="E4" s="15" t="n">
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>nps_lider_patio</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
         <v>79</v>
       </c>
-      <c r="F4" s="15" t="n"/>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>2026-06</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>nps_operador_frota</t>
         </is>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
         <v>77</v>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="E7" t="n">
         <v>79</v>
       </c>
-      <c r="E5" s="15" t="n">
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>nps_operador_frota</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
         <v>79</v>
       </c>
-      <c r="F5" s="15" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>2026-06</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>nps_outros</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
         <v>77</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="E9" t="n">
         <v>79</v>
       </c>
-      <c r="E6" s="15" t="n">
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>nps_outros</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
         <v>79</v>
       </c>
-      <c r="F6" s="15" t="n"/>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>2026-06</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>nonrev</t>
         </is>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
         <v>2.51</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="E11" t="n">
         <v>3.5</v>
       </c>
-      <c r="E7" s="15" t="n"/>
-      <c r="F7" s="15" t="n">
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>nonrev</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="n">
         <v>2.5</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="9" t="n"/>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="9" t="n"/>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="9" t="n"/>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="9" t="n"/>
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="n"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="9" t="n"/>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="9" t="n"/>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="n"/>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="9" t="n"/>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="9" t="n"/>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="9" t="n"/>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="9" t="n"/>
-      <c r="F15" s="9" t="n"/>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="9" t="n"/>
-      <c r="B16" s="9" t="n"/>
-      <c r="C16" s="9" t="n"/>
-      <c r="D16" s="9" t="n"/>
-      <c r="E16" s="9" t="n"/>
-      <c r="F16" s="9" t="n"/>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="9" t="n"/>
-      <c r="B17" s="9" t="n"/>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="9" t="n"/>
-      <c r="F17" s="9" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="9" t="n"/>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="9" t="n"/>
-      <c r="F18" s="9" t="n"/>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="9" t="n"/>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="9" t="n"/>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="9" t="n"/>
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="9" t="n"/>
-      <c r="F20" s="9" t="n"/>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="9" t="n"/>
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="9" t="n"/>
-      <c r="F21" s="9" t="n"/>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="9" t="n"/>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
-      <c r="F22" s="9" t="n"/>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="9" t="n"/>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="9" t="n"/>
-      <c r="F23" s="9" t="n"/>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="9" t="n"/>
-      <c r="B24" s="9" t="n"/>
-      <c r="C24" s="9" t="n"/>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="9" t="n"/>
-      <c r="F24" s="9" t="n"/>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="9" t="n"/>
-      <c r="B25" s="9" t="n"/>
-      <c r="C25" s="9" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="9" t="n"/>
-      <c r="F25" s="9" t="n"/>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="9" t="n"/>
-      <c r="B26" s="9" t="n"/>
-      <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="9" t="n"/>
-      <c r="F26" s="9" t="n"/>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="9" t="n"/>
-      <c r="B27" s="9" t="n"/>
-      <c r="C27" s="9" t="n"/>
-      <c r="D27" s="9" t="n"/>
-      <c r="E27" s="9" t="n"/>
-      <c r="F27" s="9" t="n"/>
-    </row>
-    <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>IMPORTANTE: Adicione 5 linhas (uma por chave) para cada novo mes ANTES de rodar o calculo.</t>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>IMPORTANTE: Adicione um bloco de linhas (uma por chave x faixa) para cada novo mes ANTES de rodar o calculo.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A29:F29"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>